<commit_message>
Update PRD: add To-Do list with 24 items (14 done, 10 pending)
</commit_message>
<xml_diff>
--- a/reference/Newsletter_Config_Overview.xlsx
+++ b/reference/Newsletter_Config_Overview.xlsx
@@ -12,6 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guardrails &amp; Filters" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Known Issues &amp; Gaps" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Schedule &amp; Process" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PRD To-Do" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -21,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -44,8 +45,16 @@
       <color rgb="00666666"/>
       <sz val="9"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00006100"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="009C5700"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -56,6 +65,18 @@
       <patternFill patternType="solid">
         <fgColor rgb="00003366"/>
         <bgColor rgb="00003366"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+        <bgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+        <bgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -77,7 +98,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -92,6 +113,18 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -3170,13 +3203,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="25" customWidth="1" min="3" max="3"/>
-    <col width="45" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="70" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3197,7 +3231,12 @@
       </c>
       <c r="D1" s="6" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="E1" s="6" t="inlineStr">
+        <is>
+          <t>Implementation Notes</t>
         </is>
       </c>
     </row>
@@ -3217,9 +3256,14 @@
           <t>Monday - Friday</t>
         </is>
       </c>
-      <c r="D2" s="7" t="inlineStr">
-        <is>
-          <t>Yes - GitHub Actions cron</t>
+      <c r="D2" s="8" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="E2" s="7" t="inlineStr">
+        <is>
+          <t>GitHub Actions cron at 1:00 UTC. Full pipeline: fetch → filter → screenshot → PDF → Telegram. Monday uses 70h lookback for Sat/Sun coverage.</t>
         </is>
       </c>
     </row>
@@ -3239,9 +3283,14 @@
           <t>Monday - Friday</t>
         </is>
       </c>
-      <c r="D3" s="7" t="inlineStr">
-        <is>
-          <t>Not yet - needs separate summary format</t>
+      <c r="D3" s="8" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="E3" s="7" t="inlineStr">
+        <is>
+          <t>GitHub Actions cron at 2:30 UTC. Text-only Telegram summary of 1st cut stories. Press release dedup (lists all publications). --mode morning-brief</t>
         </is>
       </c>
     </row>
@@ -3261,9 +3310,14 @@
           <t>Monday - Friday</t>
         </is>
       </c>
-      <c r="D4" s="7" t="inlineStr">
-        <is>
-          <t>Not yet - needs delta logic (new articles since 6:30)</t>
+      <c r="D4" s="8" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>GitHub Actions cron at 3:30 UTC. Fetches delta articles since 1st cut (6h lookback). New articles get screenshots + PDF. --mode final-cut</t>
         </is>
       </c>
     </row>
@@ -3275,17 +3329,874 @@
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>Various (next day 12PM, +2 days, +2 days, 7th day)</t>
+          <t>Various</t>
         </is>
       </c>
       <c r="C5" s="7" t="inlineStr">
         <is>
-          <t>As needed per press release</t>
-        </is>
-      </c>
-      <c r="D5" s="7" t="inlineStr">
-        <is>
-          <t>Not yet - requires tracking press releases</t>
+          <t>Per press release</t>
+        </is>
+      </c>
+      <c r="D5" s="9" t="inlineStr">
+        <is>
+          <t>TO-DO</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>Requires: (1) Press release detection, (2) Stateful tracking over 7 days, (3) 4 follow-up reports at Day+1 12PM, Day+3 11AM, Day+5 11AM, Day+7 11AM. Complex - needs database/state storage.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G25"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="35" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="70" customWidth="1" min="6" max="6"/>
+    <col width="45" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B1" s="6" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="C1" s="6" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+      <c r="D1" s="6" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="E1" s="6" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="F1" s="6" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="G1" s="6" t="inlineStr">
+        <is>
+          <t>Dependencies</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="7" t="inlineStr">
+        <is>
+          <t>1st Cut Pipeline (6:30 AM)</t>
+        </is>
+      </c>
+      <c r="C2" s="7" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="D2" s="10" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="E2" s="7" t="inlineStr">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="F2" s="7" t="inlineStr">
+        <is>
+          <t>Full pipeline: Google News RSS fetch → keyword filter → publication whitelist → dedup → Playwright screenshots → PDF report → Telegram delivery</t>
+        </is>
+      </c>
+      <c r="G2" s="7" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>Morning Brief (8:00 AM)</t>
+        </is>
+      </c>
+      <c r="C3" s="7" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="D3" s="10" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="E3" s="7" t="inlineStr">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="F3" s="7" t="inlineStr">
+        <is>
+          <t>Concise text-only Telegram summary of 1st cut stories. Press release grouping (one summary + all publications listed).</t>
+        </is>
+      </c>
+      <c r="G3" s="7" t="inlineStr">
+        <is>
+          <t>Depends on 1st Cut state file</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>Final Cut (9:00 AM)</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="D4" s="10" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="F4" s="7" t="inlineStr">
+        <is>
+          <t>Delta articles since 1st cut. 6h lookback, excludes already-reported URLs. Screenshots + PDF + Telegram for new articles only.</t>
+        </is>
+      </c>
+      <c r="G4" s="7" t="inlineStr">
+        <is>
+          <t>Depends on 1st Cut state file</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>GitHub Actions CI/CD</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="D5" s="10" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>Infra</t>
+        </is>
+      </c>
+      <c r="F5" s="7" t="inlineStr">
+        <is>
+          <t>3 cron schedules Mon-Fri (6:30, 8:00, 9:00 IST). Manual trigger with mode dropdown. Auto-commit reports to repo.</t>
+        </is>
+      </c>
+      <c r="G5" s="7" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>Telegram Bot Integration</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="D6" s="10" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="inlineStr">
+        <is>
+          <t>Delivery</t>
+        </is>
+      </c>
+      <c r="F6" s="7" t="inlineStr">
+        <is>
+          <t>Inline summary messages (categorized headlines + links) + PDF attachment. Error notifications on failure.</t>
+        </is>
+      </c>
+      <c r="G6" s="7" t="inlineStr">
+        <is>
+          <t>Bot token + Chat ID in secrets</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>Anti-Bot Screenshot Stealth</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D7" s="10" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="E7" s="7" t="inlineStr">
+        <is>
+          <t>Quality</t>
+        </is>
+      </c>
+      <c r="F7" s="7" t="inlineStr">
+        <is>
+          <t>Fake navigator.webdriver, random UA rotation (5 agents), human-like delays (1-3s), scroll simulation, blocks ads/analytics.</t>
+        </is>
+      </c>
+      <c r="G7" s="7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>PDF Clickable Links</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D8" s="10" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="E8" s="7" t="inlineStr">
+        <is>
+          <t>Quality</t>
+        </is>
+      </c>
+      <c r="F8" s="7" t="inlineStr">
+        <is>
+          <t>All headlines + URLs are clickable hyperlinks in PDF. XML-escaped for special characters (&amp;, quotes).</t>
+        </is>
+      </c>
+      <c r="G8" s="7" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="7" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>PDF Internal Navigation</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D9" s="10" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="E9" s="7" t="inlineStr">
+        <is>
+          <t>Quality</t>
+        </is>
+      </c>
+      <c r="F9" s="7" t="inlineStr">
+        <is>
+          <t>Glossary at top with anchor links to each category section. Category headers are link targets.</t>
+        </is>
+      </c>
+      <c r="G9" s="7" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>PDF Aspect Ratio Fix</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D10" s="10" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="E10" s="7" t="inlineStr">
+        <is>
+          <t>Quality</t>
+        </is>
+      </c>
+      <c r="F10" s="7" t="inlineStr">
+        <is>
+          <t>Screenshots maintain original width:height ratio. Scale to fit width, then cap height if needed.</t>
+        </is>
+      </c>
+      <c r="G10" s="7" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>Keyword Exclude Filtering</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D11" s="10" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="E11" s="7" t="inlineStr">
+        <is>
+          <t>Quality</t>
+        </is>
+      </c>
+      <c r="F11" s="7" t="inlineStr">
+        <is>
+          <t>Global excludes (cricket, sports, bollywood, lifestyle). Per-category excludes (AI hiring, jobs, etc). Blocks irrelevant noise.</t>
+        </is>
+      </c>
+      <c r="G11" s="7" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>Publication Whitelist</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D12" s="10" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="E12" s="7" t="inlineStr">
+        <is>
+          <t>Quality</t>
+        </is>
+      </c>
+      <c r="F12" s="7" t="inlineStr">
+        <is>
+          <t>~150+ whitelisted publications across 8 categories. Unknown sources dropped. Priority ranking for dedup.</t>
+        </is>
+      </c>
+      <c r="G12" s="7" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>Monday Weekend Coverage</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D13" s="10" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="E13" s="7" t="inlineStr">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="F13" s="7" t="inlineStr">
+        <is>
+          <t>70-hour lookback on Mondays (from Friday 10 AM) to cover Saturday + Sunday news.</t>
+        </is>
+      </c>
+      <c r="G13" s="7" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>TOC Column Layout Fix</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D14" s="10" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="E14" s="7" t="inlineStr">
+        <is>
+          <t>Quality</t>
+        </is>
+      </c>
+      <c r="F14" s="7" t="inlineStr">
+        <is>
+          <t>Removed Page No column. Widened headline column. No more text overlap between columns.</t>
+        </is>
+      </c>
+      <c r="G14" s="7" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="7" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>7-Day Report Retention</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D15" s="10" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="E15" s="7" t="inlineStr">
+        <is>
+          <t>Infra</t>
+        </is>
+      </c>
+      <c r="F15" s="7" t="inlineStr">
+        <is>
+          <t>Auto-cleanup of PDFs, HTMLs, and screenshots older than 7 days.</t>
+        </is>
+      </c>
+      <c r="G15" s="7" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="7" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>Coverage Dossier Automation</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D16" s="11" t="inlineStr">
+        <is>
+          <t>TO-DO</t>
+        </is>
+      </c>
+      <c r="E16" s="7" t="inlineStr">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="F16" s="7" t="inlineStr">
+        <is>
+          <t>Track press releases and auto-generate 4 follow-up coverage reports over 7 days: Day+1 (12PM), Day+3 (11AM), Day+5 (11AM), Day+7 (11AM).</t>
+        </is>
+      </c>
+      <c r="G16" s="7" t="inlineStr">
+        <is>
+          <t>Needs: press release detection logic, persistent state (DB or JSON), scheduled follow-up triggers</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="7" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>Press Release Detection</t>
+        </is>
+      </c>
+      <c r="C17" s="7" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D17" s="11" t="inlineStr">
+        <is>
+          <t>TO-DO</t>
+        </is>
+      </c>
+      <c r="E17" s="7" t="inlineStr">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="F17" s="7" t="inlineStr">
+        <is>
+          <t>Identify when an article is a press release (vs organic news). Use patterns: multiple publications same headline, 'press release' in text.</t>
+        </is>
+      </c>
+      <c r="G17" s="7" t="inlineStr">
+        <is>
+          <t>Required for Coverage Dossiers</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="7" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>Dossier State Storage</t>
+        </is>
+      </c>
+      <c r="C18" s="7" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D18" s="11" t="inlineStr">
+        <is>
+          <t>TO-DO</t>
+        </is>
+      </c>
+      <c r="E18" s="7" t="inlineStr">
+        <is>
+          <t>Infra</t>
+        </is>
+      </c>
+      <c r="F18" s="7" t="inlineStr">
+        <is>
+          <t>Persistent storage for tracking active dossiers - which PR, when it was issued, which follow-ups are pending. JSON file or SQLite.</t>
+        </is>
+      </c>
+      <c r="G18" s="7" t="inlineStr">
+        <is>
+          <t>Required for Coverage Dossiers</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="7" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>Print Article Hyperlinking</t>
+        </is>
+      </c>
+      <c r="C19" s="7" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D19" s="11" t="inlineStr">
+        <is>
+          <t>TO-DO</t>
+        </is>
+      </c>
+      <c r="E19" s="7" t="inlineStr">
+        <is>
+          <t>Quality</t>
+        </is>
+      </c>
+      <c r="F19" s="7" t="inlineStr">
+        <is>
+          <t>Process doc says print coverages should be hyperlinked within the document (internal PDF links). Currently only online links are hyperlinked externally.</t>
+        </is>
+      </c>
+      <c r="G19" s="7" t="inlineStr">
+        <is>
+          <t>Need to identify print vs online articles</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="7" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="7" t="inlineStr">
+        <is>
+          <t>Category Header Internal Hyperlinks in TOC</t>
+        </is>
+      </c>
+      <c r="C20" s="7" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D20" s="10" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="E20" s="7" t="inlineStr">
+        <is>
+          <t>Quality</t>
+        </is>
+      </c>
+      <c r="F20" s="7" t="inlineStr">
+        <is>
+          <t>TOC category headers should link to their section. Currently done via glossary anchor links.</t>
+        </is>
+      </c>
+      <c r="G20" s="7" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="7" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="7" t="inlineStr">
+        <is>
+          <t>Negative Keyword Expansion</t>
+        </is>
+      </c>
+      <c r="C21" s="7" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="D21" s="11" t="inlineStr">
+        <is>
+          <t>TO-DO</t>
+        </is>
+      </c>
+      <c r="E21" s="7" t="inlineStr">
+        <is>
+          <t>Quality</t>
+        </is>
+      </c>
+      <c r="F21" s="7" t="inlineStr">
+        <is>
+          <t>Add more exclude patterns as false positives are identified. Consider regex-based exclusion for complex patterns.</t>
+        </is>
+      </c>
+      <c r="G21" s="7" t="inlineStr">
+        <is>
+          <t>Ongoing tuning</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="7" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="7" t="inlineStr">
+        <is>
+          <t>Article Body Filtering (NLP)</t>
+        </is>
+      </c>
+      <c r="C22" s="7" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="D22" s="11" t="inlineStr">
+        <is>
+          <t>TO-DO</t>
+        </is>
+      </c>
+      <c r="E22" s="7" t="inlineStr">
+        <is>
+          <t>Quality</t>
+        </is>
+      </c>
+      <c r="F22" s="7" t="inlineStr">
+        <is>
+          <t>Currently filters by headline only. Reading article body + NLP relevance scoring would improve accuracy significantly.</t>
+        </is>
+      </c>
+      <c r="G22" s="7" t="inlineStr">
+        <is>
+          <t>Requires: article text scraping + NLP library (high complexity)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="7" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="7" t="inlineStr">
+        <is>
+          <t>Multiple Edition Handling</t>
+        </is>
+      </c>
+      <c r="C23" s="7" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="D23" s="11" t="inlineStr">
+        <is>
+          <t>TO-DO</t>
+        </is>
+      </c>
+      <c r="E23" s="7" t="inlineStr">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="F23" s="7" t="inlineStr">
+        <is>
+          <t>Process doc says 'keep single edition for stories under other sections'. Need smarter dedup that identifies same story across editions.</t>
+        </is>
+      </c>
+      <c r="G23" s="7" t="inlineStr">
+        <is>
+          <t>Enhancement to dedup logic</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="7" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="7" t="inlineStr">
+        <is>
+          <t>Telegram Bot Commands</t>
+        </is>
+      </c>
+      <c r="C24" s="7" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="D24" s="11" t="inlineStr">
+        <is>
+          <t>TO-DO</t>
+        </is>
+      </c>
+      <c r="E24" s="7" t="inlineStr">
+        <is>
+          <t>Delivery</t>
+        </is>
+      </c>
+      <c r="F24" s="7" t="inlineStr">
+        <is>
+          <t>Add /generate, /status, /brief slash commands so users can trigger reports on-demand from Telegram.</t>
+        </is>
+      </c>
+      <c r="G24" s="7" t="inlineStr">
+        <is>
+          <t>Optional enhancement</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="7" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="7" t="inlineStr">
+        <is>
+          <t>Email Delivery Option</t>
+        </is>
+      </c>
+      <c r="C25" s="7" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="D25" s="11" t="inlineStr">
+        <is>
+          <t>TO-DO</t>
+        </is>
+      </c>
+      <c r="E25" s="7" t="inlineStr">
+        <is>
+          <t>Delivery</t>
+        </is>
+      </c>
+      <c r="F25" s="7" t="inlineStr">
+        <is>
+          <t>Some stakeholders may prefer email. Add optional SMTP delivery alongside Telegram.</t>
+        </is>
+      </c>
+      <c r="G25" s="7" t="inlineStr">
+        <is>
+          <t>Optional - if requested</t>
         </is>
       </c>
     </row>

</xml_diff>